<commit_message>
Corrida | SFE-REC | 2026-04-07 08:25:00.720692
</commit_message>
<xml_diff>
--- a/indicadores/SFE-REC_out.xlsx
+++ b/indicadores/SFE-REC_out.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Correlograma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Correlograma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -49,7 +50,7 @@
     <t xml:space="preserve">Sector</t>
   </si>
   <si>
-    <t xml:space="preserve">Recursos y gastos del sector público de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Recursos y gastos del sector público</t>
   </si>
   <si>
     <t xml:space="preserve">Modelo</t>
@@ -103,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">23/02/2026</t>
+    <t xml:space="preserve">07/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">ysonder</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1571,6 +1572,63 @@
   </si>
   <si>
     <t xml:space="preserve">2030.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias de las series incluidas en la hoja Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_normal | serie original con 12 forecasts obtenidos del mejor modelo ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_optimista | serie original con 12 forecasts, intervalo y límite optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_pesimista | serie original con 12 forecasts, intervalo y límite pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_d16 | salida D16 del X13-ARIMA-SEATS con los factores estacionales de la serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_c17 | salida C17 del X13-ARIMA-SEATS con pesos del irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_d12 | salida D12 del X13-ARIMA-SEATS con el componente tendencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_129600 | tendencia HP de largo plazo con un lambda de 129.600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_200 | suavizado con filtro HP usando lambda de 200, sirve para determinar PG automáticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e_ajustada | serie ajustada por estacionalidad usando el mejor modelo (LOG o NIV según el caso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_filtrada | serie ajustada por estacionalidad y corregida por irregularidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final | serie f_filtrada con o sin suavizado 2x2 según el caso (es la vieja española)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final_fct_normal | a_original_fct ajustada por D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_tcml | tasas de cambio mensual logarítmicas de la serie g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_var_interanual | variaciones interanuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_var_mensual | variaciones mensuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_irregular | g_final/d_d12 componente irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i_dt | g_final/d_hp_129600 desvíos respecto de la tendencia</t>
   </si>
   <si>
     <t xml:space="preserve">Coeficientes de correlación de TCML del ICA-SFE y serie específica</t>
@@ -2167,7 +2225,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.497905102340129</v>
+        <v>0.498087693824228</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2225,7 +2283,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.247909490936334</v>
+        <v>0.248091350739138</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2295,7 +2353,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0000311154891106025</v>
+        <v>0.0000290191482931125</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2325,7 +2383,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000149256384813528</v>
+        <v>0.000144580323616516</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -28125,200 +28183,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>519</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>519</v>
-      </c>
-      <c r="B2" s="1"/>
+        <v>520</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3"/>
-      <c r="B3" s="1"/>
+      <c r="A3" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>520</v>
-      </c>
-      <c r="B4" s="1"/>
+        <v>522</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>521</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>0.145823861492582</v>
+        <v>523</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>522</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0.15460135483207</v>
+        <v>524</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>523</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>0.178471288175489</v>
+        <v>525</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>524</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>0.182528579072194</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>525</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>0.170171080696689</v>
+        <v>527</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>526</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>0.217448271105859</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>527</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>0.263192379441991</v>
+        <v>529</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>528</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>0.329924072538795</v>
+        <v>530</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>529</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>0.471065080746154</v>
+        <v>531</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>530</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>0.497905102340129</v>
+        <v>532</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>531</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>0.365692741297959</v>
+        <v>533</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>532</v>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>0.285944586087619</v>
+        <v>534</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>533</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>0.271925220711846</v>
+        <v>535</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>534</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>0.260326415216264</v>
+        <v>536</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>535</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>0.240283413890565</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>536</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>0.182011344464871</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
         <v>537</v>
       </c>
-      <c r="B21" s="1" t="n">
-        <v>0.128097697152617</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>538</v>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>0.123969273249369</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>539</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>0.117741679721542</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="1"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="1"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="1"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="1"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="1"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28326,235 +28282,210 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC12BB18-D94A-42B0-8417-CACC7D53CBA2}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D90DEEE-34B0-4CD4-A0CF-87949F5D9E97}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{573756CF-146F-470B-A04D-3F26964E8029}"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>539</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>540</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0.145604139480452</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>541</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0.152897188975961</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>542</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.17751236353055</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>543</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>0.182466820077314</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>544</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>0.16972034930296</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>545</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>0.218058469041816</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>546</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0.263320549062641</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>547</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.32797930486816</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>548</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0.469799749742905</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>549</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.498087693824228</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>550</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0.36615973399947</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>551</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0.287262385522104</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>552</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>0.274598316577224</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>553</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>0.261556493561946</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>554</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>0.238995466862658</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>555</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>0.181740273409998</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>556</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>0.129026007750762</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>557</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>0.123791308315452</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>558</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>0.117639251908169</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-REC | 2026-06-17 11:59:03.455942
</commit_message>
<xml_diff>
--- a/indicadores/SFE-REC_out.xlsx
+++ b/indicadores/SFE-REC_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="561">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">26/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2193,9 +2199,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2206,7 +2216,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2220,12 +2230,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.503255885804954</v>
+        <v>0.50242810943789</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2236,7 +2246,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2264,7 +2274,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2278,12 +2288,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.253266486597329</v>
+        <v>0.252434005153333</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2306,7 +2316,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2320,7 +2330,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2334,7 +2344,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2348,12 +2358,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.000046838219706666</v>
+        <v>0.0000416798070422152</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2364,7 +2374,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2378,12 +2388,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000160962501841104</v>
+        <v>0.000187536282126564</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2526,10 +2536,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2542,10 +2552,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2569,66 +2579,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>60.908215637091</v>
@@ -2681,7 +2691,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>61.580050524226</v>
@@ -2738,7 +2748,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>59.9522682230437</v>
@@ -2795,7 +2805,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>61.7946144578847</v>
@@ -2852,7 +2862,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>76.7396091551446</v>
@@ -2909,7 +2919,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>97.0733683795534</v>
@@ -2966,7 +2976,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>69.3589737152524</v>
@@ -3023,7 +3033,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>63.0591362200402</v>
@@ -3080,7 +3090,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>74.7382658542811</v>
@@ -3137,7 +3147,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>56.7717322888232</v>
@@ -3194,7 +3204,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>70.1218825471414</v>
@@ -3251,7 +3261,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>73.8315051541047</v>
@@ -3308,7 +3318,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>79.2578531538842</v>
@@ -3367,7 +3377,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>70.4061159402138</v>
@@ -3426,7 +3436,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>69.7884085270014</v>
@@ -3485,7 +3495,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>67.1935920937369</v>
@@ -3544,7 +3554,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>66.7426812241839</v>
@@ -3603,7 +3613,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>59.5686269601538</v>
@@ -3662,7 +3672,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>71.3227605342928</v>
@@ -3721,7 +3731,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>58.8092220794395</v>
@@ -3780,7 +3790,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>72.9149604617445</v>
@@ -3839,7 +3849,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>80.0555136650045</v>
@@ -3898,7 +3908,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>94.8435598724428</v>
@@ -3957,7 +3967,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>90.1901892768105</v>
@@ -4016,7 +4026,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>73.5528295537216</v>
@@ -4075,7 +4085,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>85.5523195630849</v>
@@ -4134,7 +4144,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>73.5571197538839</v>
@@ -4193,7 +4203,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>77.3521823038247</v>
@@ -4252,7 +4262,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>87.4349634201883</v>
@@ -4311,7 +4321,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>84.9856251416553</v>
@@ -4370,7 +4380,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>70.5275423959374</v>
@@ -4429,7 +4439,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>62.7451756601945</v>
@@ -4488,7 +4498,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>77.5453222505169</v>
@@ -4547,7 +4557,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>79.5856930650873</v>
@@ -4606,7 +4616,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>68.3590378401964</v>
@@ -4665,7 +4675,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>111.891279341244</v>
@@ -4724,7 +4734,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>70.5414758036367</v>
@@ -4783,7 +4793,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>77.5150425996004</v>
@@ -4842,7 +4852,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>60.6426810274109</v>
@@ -4901,7 +4911,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>61.1996216287404</v>
@@ -4960,7 +4970,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>73.6429353329553</v>
@@ -5019,7 +5029,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>65.9820766785538</v>
@@ -5078,7 +5088,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>79.1900798519488</v>
@@ -5137,7 +5147,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>62.1420689204317</v>
@@ -5196,7 +5206,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>55.7605640053723</v>
@@ -5255,7 +5265,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>70.1610970702823</v>
@@ -5314,7 +5324,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>67.5046738290354</v>
@@ -5373,7 +5383,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>51.7891274034868</v>
@@ -5432,7 +5442,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>57.4344486327466</v>
@@ -5491,7 +5501,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>67.4318820858955</v>
@@ -5550,7 +5560,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>58.0854693784526</v>
@@ -5609,7 +5619,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>67.3826806661377</v>
@@ -5668,7 +5678,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>75.7247348415218</v>
@@ -5727,7 +5737,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>67.1502183392149</v>
@@ -5786,7 +5796,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>70.023233233683</v>
@@ -5845,7 +5855,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>69.4057439891169</v>
@@ -5904,7 +5914,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>59.3240500396649</v>
@@ -5963,7 +5973,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>56.0502892400782</v>
@@ -6022,7 +6032,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>80.3780534966032</v>
@@ -6081,7 +6091,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>59.0874522787738</v>
@@ -6140,7 +6150,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>56.8074529796469</v>
@@ -6199,7 +6209,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>66.6980426696578</v>
@@ -6258,7 +6268,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>88.0299443339664</v>
@@ -6317,7 +6327,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>81.9723840165564</v>
@@ -6376,7 +6386,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>79.8891012528117</v>
@@ -6435,7 +6445,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>80.0792475678922</v>
@@ -6494,7 +6504,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>84.1584320495728</v>
@@ -6553,7 +6563,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>76.6421803077947</v>
@@ -6612,7 +6622,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>71.2101595871925</v>
@@ -6671,7 +6681,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>78.3529475548963</v>
@@ -6730,7 +6740,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>80.1587023245876</v>
@@ -6789,7 +6799,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>63.8941641214641</v>
@@ -6848,7 +6858,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>69.9168012879555</v>
@@ -6907,7 +6917,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>77.7552177184693</v>
@@ -6966,7 +6976,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>74.7723124472717</v>
@@ -7025,7 +7035,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>79.4523341732934</v>
@@ -7084,7 +7094,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>85.5090179766211</v>
@@ -7143,7 +7153,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>86.6318190847228</v>
@@ -7202,7 +7212,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>91.7150315663078</v>
@@ -7261,7 +7271,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>83.7546849324324</v>
@@ -7320,7 +7330,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>75.8411746753517</v>
@@ -7379,7 +7389,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>79.8239043683697</v>
@@ -7438,7 +7448,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>84.359841683417</v>
@@ -7497,7 +7507,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>68.5574275783601</v>
@@ -7556,7 +7566,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>70.7575383675003</v>
@@ -7615,7 +7625,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>78.2466618768148</v>
@@ -7674,7 +7684,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>71.7714876686931</v>
@@ -7733,7 +7743,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>76.7348973534154</v>
@@ -7792,7 +7802,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>80.100218567988</v>
@@ -7851,7 +7861,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>85.1181796158874</v>
@@ -7910,7 +7920,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>83.0454239843793</v>
@@ -7969,7 +7979,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>78.6100132031816</v>
@@ -8028,7 +8038,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>71.7788547245143</v>
@@ -8087,7 +8097,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>75.6990539289697</v>
@@ -8146,7 +8156,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>85.4809927153223</v>
@@ -8205,7 +8215,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>99.7594290707993</v>
@@ -8264,7 +8274,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>90.3738820011741</v>
@@ -8323,7 +8333,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>87.4685212945033</v>
@@ -8382,7 +8392,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>73.5072595678171</v>
@@ -8441,7 +8451,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>89.8091519193775</v>
@@ -8500,7 +8510,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>84.9946258588306</v>
@@ -8559,7 +8569,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>87.2435286604889</v>
@@ -8618,7 +8628,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>94.1552701555462</v>
@@ -8677,7 +8687,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>79.6218078483185</v>
@@ -8736,7 +8746,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>78.7209721209145</v>
@@ -8795,7 +8805,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>84.3792435166703</v>
@@ -8854,7 +8864,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>84.4658515289066</v>
@@ -8913,7 +8923,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>72.4579681603551</v>
@@ -8972,7 +8982,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>78.1349411633508</v>
@@ -9031,7 +9041,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>79.392880503088</v>
@@ -9090,7 +9100,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>71.1006223633449</v>
@@ -9149,7 +9159,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>76.6499337544855</v>
@@ -9208,7 +9218,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>85.3873288720018</v>
@@ -9267,7 +9277,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>84.8998521457381</v>
@@ -9326,7 +9336,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>85.1167790905518</v>
@@ -9385,7 +9395,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>74.7402218736597</v>
@@ -9444,7 +9454,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>69.7098993343295</v>
@@ -9503,7 +9513,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>73.2983451665455</v>
@@ -9562,7 +9572,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>71.9889374582806</v>
@@ -9621,7 +9631,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>46.0678368477303</v>
@@ -9680,7 +9690,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>57.058111305018</v>
@@ -9739,7 +9749,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>56.8364577737455</v>
@@ -9798,7 +9808,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>52.6493598379911</v>
@@ -9857,7 +9867,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>52.5236627562416</v>
@@ -9916,7 +9926,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>59.4033654367252</v>
@@ -9975,7 +9985,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>55.5379293931647</v>
@@ -10034,7 +10044,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>60.1717424447995</v>
@@ -10093,7 +10103,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>53.6355436619042</v>
@@ -10152,7 +10162,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>51.0928494327459</v>
@@ -10211,7 +10221,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>59.4779665320163</v>
@@ -10270,7 +10280,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>60.3588966441247</v>
@@ -10329,7 +10339,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>53.610451919562</v>
@@ -10388,7 +10398,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>63.5877300251372</v>
@@ -10447,7 +10457,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>52.4151756593675</v>
@@ -10506,7 +10516,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>48.2213668747725</v>
@@ -10565,7 +10575,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>55.2284773998603</v>
@@ -10624,7 +10634,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>61.9447975730277</v>
@@ -10683,7 +10693,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>55.8045879240194</v>
@@ -10742,7 +10752,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>54.2990351385357</v>
@@ -10801,7 +10811,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>53.3076016869343</v>
@@ -10860,7 +10870,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>73.2468801256804</v>
@@ -10919,7 +10929,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>73.5526534368707</v>
@@ -10978,7 +10988,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>81.1388160478511</v>
@@ -11037,7 +11047,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>66.7442267142617</v>
@@ -11096,7 +11106,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>63.5136993679848</v>
@@ -11155,7 +11165,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>66.8927232733957</v>
@@ -11214,7 +11224,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>82.6501005462773</v>
@@ -11273,7 +11283,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>73.2945987436672</v>
@@ -11332,7 +11342,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>75.2670536062459</v>
@@ -11391,7 +11401,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>74.7709792124781</v>
@@ -11450,7 +11460,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>68.5315771941142</v>
@@ -11509,7 +11519,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>83.6943285898011</v>
@@ -11568,7 +11578,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>73.2744287297783</v>
@@ -11627,7 +11637,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>81.5549335981247</v>
@@ -11686,7 +11696,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>73.7015628989377</v>
@@ -11745,7 +11755,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>75.0236414517588</v>
@@ -11804,7 +11814,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>80.4307140495308</v>
@@ -11863,7 +11873,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>86.3747512323693</v>
@@ -11922,7 +11932,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>67.4117799762781</v>
@@ -11981,7 +11991,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>79.654609157932</v>
@@ -12040,7 +12050,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>82.8028912630047</v>
@@ -12099,7 +12109,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>87.057962478428</v>
@@ -12158,7 +12168,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>84.3680115839347</v>
@@ -12217,7 +12227,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>75.8343372254624</v>
@@ -12276,7 +12286,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>79.6455023728216</v>
@@ -12335,7 +12345,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>82.4999531030183</v>
@@ -12394,7 +12404,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>84.3449109704511</v>
@@ -12453,7 +12463,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>73.2876913700384</v>
@@ -12512,7 +12522,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>76.3824882265344</v>
@@ -12571,7 +12581,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>97.0393367539515</v>
@@ -12630,7 +12640,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>75.181542365012</v>
@@ -12689,7 +12699,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>81.2753567900812</v>
@@ -12748,7 +12758,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>87.9334716471331</v>
@@ -12807,7 +12817,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>92.2094009946976</v>
@@ -12866,7 +12876,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>93.0692502529268</v>
@@ -12925,7 +12935,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>83.9866422529311</v>
@@ -12984,7 +12994,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>88.5604511236838</v>
@@ -13043,7 +13053,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>88.5440437625363</v>
@@ -13102,7 +13112,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>90.4156479471919</v>
@@ -13161,7 +13171,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>77.8895787118718</v>
@@ -13220,7 +13230,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>84.6227590727579</v>
@@ -13279,7 +13289,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>102.862295059307</v>
@@ -13338,7 +13348,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>81.9133042659247</v>
@@ -13397,7 +13407,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>87.4682162713906</v>
@@ -13456,7 +13466,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>91.5407906461947</v>
@@ -13515,7 +13525,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>102.152371713638</v>
@@ -13574,7 +13584,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>99.4680045999919</v>
@@ -13633,7 +13643,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>96.3284247397764</v>
@@ -13692,7 +13702,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>97.7525975756168</v>
@@ -13751,7 +13761,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>100.254628140161</v>
@@ -13810,7 +13820,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>106.790932251231</v>
@@ -13869,7 +13879,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>94.1027048022173</v>
@@ -13928,7 +13938,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>100.230635954985</v>
@@ -13987,7 +13997,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>117.878818353316</v>
@@ -14046,7 +14056,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>89.4453157027337</v>
@@ -14105,7 +14115,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>98.5815110705265</v>
@@ -14164,7 +14174,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>104.588038337289</v>
@@ -14223,7 +14233,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>106.575043815146</v>
@@ -14282,7 +14292,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>110.02043433483</v>
@@ -14341,7 +14351,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>104.687331835651</v>
@@ -14400,7 +14410,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>102.884545376569</v>
@@ -14459,7 +14469,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>99.785248646306</v>
@@ -14518,7 +14528,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>98.3191275771912</v>
@@ -14577,7 +14587,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>89.9934139877799</v>
@@ -14636,7 +14646,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>102.040794205578</v>
@@ -14695,7 +14705,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>108.219498508479</v>
@@ -14754,7 +14764,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>85.6923291130906</v>
@@ -14813,7 +14823,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>99.4263307698801</v>
@@ -14872,7 +14882,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>93.8232174838228</v>
@@ -14931,7 +14941,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>106.706374811371</v>
@@ -14990,7 +15000,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>104.592878512603</v>
@@ -15049,7 +15059,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>102.741588201261</v>
@@ -15108,7 +15118,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>111.138505648011</v>
@@ -15167,7 +15177,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>100.579242874937</v>
@@ -15226,7 +15236,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>101.499942044821</v>
@@ -15285,7 +15295,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>88.4243370677871</v>
@@ -15344,7 +15354,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>91.3415214243162</v>
@@ -15403,7 +15413,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>117.077111698844</v>
@@ -15462,7 +15472,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>109.460086549308</v>
@@ -15521,7 +15531,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>128.864141614791</v>
@@ -15580,7 +15590,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>127.92964737898</v>
@@ -15639,7 +15649,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>129.617469785827</v>
@@ -15698,7 +15708,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>131.202440120432</v>
@@ -15757,7 +15767,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>125.273432595285</v>
@@ -15816,7 +15826,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>121.627367185041</v>
@@ -15875,7 +15885,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>118.851697820774</v>
@@ -15934,7 +15944,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>124.758390927586</v>
@@ -15993,7 +16003,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>117.281762492161</v>
@@ -16052,7 +16062,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>121.709543956811</v>
@@ -16111,7 +16121,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>134.80868523675</v>
@@ -16170,7 +16180,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>112.512114190825</v>
@@ -16229,7 +16239,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>122.438700276356</v>
@@ -16288,7 +16298,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>134.262624599472</v>
@@ -16347,7 +16357,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>148.025230843731</v>
@@ -16406,7 +16416,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>141.169859453861</v>
@@ -16465,7 +16475,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>130.851309269567</v>
@@ -16524,7 +16534,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>139.759855601649</v>
@@ -16583,7 +16593,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>133.224575401522</v>
@@ -16642,7 +16652,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>134.824445821102</v>
@@ -16701,7 +16711,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>121.653960529104</v>
@@ -16760,7 +16770,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>126.149968648238</v>
@@ -16819,7 +16829,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>138.423843885239</v>
@@ -16878,7 +16888,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>126.924875249057</v>
@@ -16937,7 +16947,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>120.826628751903</v>
@@ -16996,7 +17006,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>136.885453087214</v>
@@ -17055,7 +17065,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>137.036452120855</v>
@@ -17114,7 +17124,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>130.787935452228</v>
@@ -17173,7 +17183,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>125.854415206171</v>
@@ -17232,7 +17242,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>126.543478491896</v>
@@ -17291,7 +17301,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>132.202038185303</v>
@@ -17350,7 +17360,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>138.496031459386</v>
@@ -17409,7 +17419,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>130.65564157072</v>
@@ -17468,7 +17478,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>138.610721936559</v>
@@ -17527,7 +17537,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>155.165774747856</v>
@@ -17586,7 +17596,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>139.174861063213</v>
@@ -17645,7 +17655,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>148.663545833441</v>
@@ -17704,7 +17714,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>147.429910537389</v>
@@ -17763,7 +17773,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>160.780506082671</v>
@@ -17822,7 +17832,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>141.812831188301</v>
@@ -17881,7 +17891,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>148.775903096039</v>
@@ -17940,7 +17950,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>153.344327160745</v>
@@ -17999,7 +18009,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>140.718775391458</v>
@@ -18058,7 +18068,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>154.019129859815</v>
@@ -18117,7 +18127,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>145.759903348614</v>
@@ -18176,7 +18186,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>139.729396681939</v>
@@ -18235,7 +18245,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>166.609668996424</v>
@@ -18294,7 +18304,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>122.755940305729</v>
@@ -18353,7 +18363,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>141.413763817478</v>
@@ -18412,7 +18422,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>134.682575892957</v>
@@ -18471,7 +18481,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>156.13425378031</v>
@@ -18530,7 +18540,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>141.40013248785</v>
@@ -18589,7 +18599,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>143.546340593526</v>
@@ -18648,7 +18658,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>156.349964812799</v>
@@ -18707,7 +18717,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>140.877117179411</v>
@@ -18766,7 +18776,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>147.125315024315</v>
@@ -18825,7 +18835,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>141.623664579178</v>
@@ -18884,7 +18894,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>132.900857949694</v>
@@ -18943,7 +18953,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>155.824420928943</v>
@@ -19002,7 +19012,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>131.47974668115</v>
@@ -19061,7 +19071,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>156.292555570365</v>
@@ -19120,7 +19130,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>146.024878191581</v>
@@ -19179,7 +19189,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>161.802595519576</v>
@@ -19238,7 +19248,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>149.403126289127</v>
@@ -19297,7 +19307,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>147.489851405405</v>
@@ -19356,7 +19366,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>148.845144014014</v>
@@ -19415,7 +19425,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>143.909588856616</v>
@@ -19474,7 +19484,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>156.182442848749</v>
@@ -19533,7 +19543,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>150.670031174131</v>
@@ -19592,7 +19602,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>136.376001090417</v>
@@ -19651,7 +19661,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>168.516883039073</v>
@@ -19710,7 +19720,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>148.31091738146</v>
@@ -19769,7 +19779,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>162.358793643755</v>
@@ -19828,7 +19838,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>139.516297923181</v>
@@ -19887,7 +19897,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>157.874124803267</v>
@@ -19946,7 +19956,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>146.933184462614</v>
@@ -20005,7 +20015,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>148.319721627461</v>
@@ -20064,7 +20074,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>162.042004060776</v>
@@ -20123,7 +20133,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>143.16574889132</v>
@@ -20182,7 +20192,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>154.743467299379</v>
@@ -20241,7 +20251,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>162.718708447896</v>
@@ -20300,7 +20310,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>156.939648076185</v>
@@ -20359,7 +20369,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>177.334595348609</v>
@@ -20418,7 +20428,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>133.579725895037</v>
@@ -20477,7 +20487,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>153.3352296795</v>
@@ -20536,7 +20546,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>148.716252683841</v>
@@ -20595,7 +20605,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>171.744044416365</v>
@@ -20654,7 +20664,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>157.751030798625</v>
@@ -20713,7 +20723,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>162.190143126223</v>
@@ -20772,7 +20782,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>167.751141905986</v>
@@ -20831,7 +20841,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>154.191384809262</v>
@@ -20890,7 +20900,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>161.836683748292</v>
@@ -20949,7 +20959,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>158.638385839956</v>
@@ -21008,7 +21018,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>151.85196095576</v>
@@ -21067,7 +21077,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>164.35000049841</v>
@@ -21126,7 +21136,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>137.574124789569</v>
@@ -21185,7 +21195,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>149.029269951035</v>
@@ -21244,7 +21254,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>164.120949622351</v>
@@ -21303,7 +21313,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>173.046111714172</v>
@@ -21362,7 +21372,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>150.042236169212</v>
@@ -21421,7 +21431,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>163.74391824386</v>
@@ -21480,7 +21490,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>165.440462245396</v>
@@ -21539,7 +21549,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>144.201607300226</v>
@@ -21598,7 +21608,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>161.322197743055</v>
@@ -21657,7 +21667,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>156.177876090747</v>
@@ -21716,7 +21726,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>136.944332288135</v>
@@ -21775,7 +21785,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>166.38482591886</v>
@@ -21834,7 +21844,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>128.645259666901</v>
@@ -21893,7 +21903,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>143.402106390566</v>
@@ -21952,7 +21962,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>137.225285231644</v>
@@ -22011,7 +22021,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>142.987100634546</v>
@@ -22070,7 +22080,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>132.723859190404</v>
@@ -22129,7 +22139,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>143.38417880331</v>
@@ -22188,7 +22198,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>147.147154899028</v>
@@ -22247,7 +22257,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>137.490441360114</v>
@@ -22306,7 +22316,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>147.901017101719</v>
@@ -22365,7 +22375,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>145.789650885926</v>
@@ -22424,7 +22434,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>133.11729088877</v>
@@ -22483,7 +22493,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>163.981058291002</v>
@@ -22542,7 +22552,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>117.936543958601</v>
@@ -22601,7 +22611,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>110.529917023447</v>
@@ -22660,7 +22670,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>129.116747665231</v>
@@ -22719,7 +22729,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>148.571378361387</v>
@@ -22778,7 +22788,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>149.773114689698</v>
@@ -22837,7 +22847,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>149.352873971863</v>
@@ -22896,7 +22906,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>148.544840439766</v>
@@ -22955,7 +22965,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>142.030805230753</v>
@@ -23014,7 +23024,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>153.327989750357</v>
@@ -23073,7 +23083,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>138.602886572863</v>
@@ -23132,7 +23142,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>136.562006218419</v>
@@ -23191,7 +23201,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>160.935836114426</v>
@@ -23250,7 +23260,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>134.67349506548</v>
@@ -23309,7 +23319,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>145.118926039752</v>
@@ -23368,7 +23378,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>145.378895671755</v>
@@ -23427,7 +23437,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>154.583572141249</v>
@@ -23486,7 +23496,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>144.607164999984</v>
@@ -23545,7 +23555,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>155.717214857666</v>
@@ -23604,7 +23614,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>157.560305006351</v>
@@ -23663,7 +23673,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>145.287751010011</v>
@@ -23722,7 +23732,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>157.31196570628</v>
@@ -23781,7 +23791,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>154.550715660554</v>
@@ -23840,7 +23850,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>148.333603262448</v>
@@ -23899,7 +23909,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>179.884658451763</v>
@@ -23958,7 +23968,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>134.68423050346</v>
@@ -24017,7 +24027,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>154.195938348104</v>
@@ -24076,7 +24086,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>154.606047440327</v>
@@ -24135,7 +24145,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>162.280402155235</v>
@@ -24194,7 +24204,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>155.326321199884</v>
@@ -24253,7 +24263,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>145.649386746486</v>
@@ -24312,7 +24322,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>152.881153855615</v>
@@ -24371,7 +24381,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>142.654049440622</v>
@@ -24430,7 +24440,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>141.294826641208</v>
@@ -24489,7 +24499,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>140.21562682808</v>
@@ -24548,7 +24558,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>147.022666277926</v>
@@ -24607,7 +24617,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>157.151287596023</v>
@@ -24666,7 +24676,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>125.40576635988</v>
@@ -24725,7 +24735,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>135.947167388536</v>
@@ -24784,7 +24794,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>137.849884726799</v>
@@ -24843,7 +24853,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>148.185388852607</v>
@@ -24902,7 +24912,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>147.424127360812</v>
@@ -24961,7 +24971,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>150.604195852151</v>
@@ -25020,7 +25030,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>146.491727599502</v>
@@ -25079,7 +25089,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>147.999883726462</v>
@@ -25138,7 +25148,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>137.315101852657</v>
@@ -25197,7 +25207,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>122.608075591022</v>
@@ -25256,7 +25266,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>130.012348742956</v>
@@ -25315,7 +25325,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>158.568074141782</v>
@@ -25374,7 +25384,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>124.444916627879</v>
@@ -25433,7 +25443,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>124.586590687026</v>
@@ -25492,7 +25502,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>125.91920906786</v>
@@ -25551,7 +25561,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>133.389646991025</v>
@@ -25610,7 +25620,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>123.866726404856</v>
@@ -25669,7 +25679,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>132.63361141987</v>
@@ -25728,7 +25738,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>132.482093957503</v>
@@ -25787,7 +25797,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>126.264298145061</v>
@@ -25846,7 +25856,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>134.026912127304</v>
@@ -25905,7 +25915,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>129.32321737983</v>
@@ -25964,7 +25974,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>133.509454728399</v>
@@ -26023,7 +26033,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>192.166539258414</v>
@@ -26082,7 +26092,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>117.5501077083</v>
@@ -26141,7 +26151,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>129.844463634689</v>
@@ -26200,7 +26210,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B402" s="2" t="n">
         <v>134.561196283546</v>
@@ -26259,7 +26269,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B403" s="2" t="n">
         <v>146.96942796863</v>
@@ -26318,7 +26328,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B404" s="2" t="n">
         <v>144.043207386532</v>
@@ -26377,7 +26387,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B405" s="2" t="n">
         <v>148.285565284862</v>
@@ -26436,7 +26446,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B406" s="2" t="n">
         <v>146.324252558576</v>
@@ -26495,7 +26505,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B407" s="2" t="n">
         <v>147.855102977384</v>
@@ -26554,7 +26564,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B408" s="2" t="n">
         <v>133.141108713634</v>
@@ -26613,7 +26623,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B409" s="2" t="n">
         <v>141.557461085409</v>
@@ -26672,7 +26682,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B410" s="2" t="n">
         <v>147.435599791423</v>
@@ -26731,7 +26741,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B411" s="2" t="n">
         <v>192.07880437189</v>
@@ -26790,7 +26800,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B412" s="2" t="n">
         <v>120.603485896746</v>
@@ -26849,7 +26859,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3" t="n">
@@ -26882,7 +26892,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3" t="n">
@@ -26915,7 +26925,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3" t="n">
@@ -26948,7 +26958,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3" t="n">
@@ -26981,7 +26991,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3" t="n">
@@ -27014,7 +27024,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3" t="n">
@@ -27047,7 +27057,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3" t="n">
@@ -27080,7 +27090,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3" t="n">
@@ -27113,7 +27123,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3" t="n">
@@ -27146,7 +27156,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3" t="n">
@@ -27179,7 +27189,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3" t="n">
@@ -27212,7 +27222,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3" t="n">
@@ -27245,7 +27255,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -27268,7 +27278,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -27291,7 +27301,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -27314,7 +27324,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -27337,7 +27347,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -27360,7 +27370,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -27383,7 +27393,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -27406,7 +27416,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -27429,7 +27439,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27452,7 +27462,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27475,7 +27485,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27498,7 +27508,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27521,7 +27531,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27544,7 +27554,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27567,7 +27577,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27590,7 +27600,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27613,7 +27623,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27636,7 +27646,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27659,7 +27669,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27682,7 +27692,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27705,7 +27715,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27728,7 +27738,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27751,7 +27761,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27774,7 +27784,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27797,7 +27807,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27820,7 +27830,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27843,7 +27853,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27866,7 +27876,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -27889,7 +27899,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -27912,7 +27922,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -27935,7 +27945,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -27958,7 +27968,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -27981,7 +27991,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -28004,7 +28014,7 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B458" s="2"/>
       <c r="C458" s="3"/>
@@ -28027,7 +28037,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B459" s="2"/>
       <c r="C459" s="3"/>
@@ -28050,7 +28060,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B460" s="2"/>
       <c r="C460" s="3"/>
@@ -28073,7 +28083,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B461" s="2"/>
       <c r="C461" s="3"/>
@@ -28096,7 +28106,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B462" s="2"/>
       <c r="C462" s="3"/>
@@ -28119,7 +28129,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B463" s="2"/>
       <c r="C463" s="3"/>
@@ -28142,7 +28152,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B464" s="2"/>
       <c r="C464" s="3"/>
@@ -28165,7 +28175,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B465" s="2"/>
       <c r="C465" s="3"/>
@@ -28188,7 +28198,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B466" s="2"/>
       <c r="C466" s="3"/>
@@ -28211,7 +28221,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B467" s="2"/>
       <c r="C467" s="3"/>
@@ -28234,7 +28244,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B468" s="2"/>
       <c r="C468" s="3"/>
@@ -28257,7 +28267,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B469" s="2"/>
       <c r="C469" s="3"/>
@@ -28291,97 +28301,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -28405,7 +28415,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -28415,160 +28425,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.140488675307005</v>
+        <v>0.13828454165403</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.148694314777076</v>
+        <v>0.145368691206774</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.179688848483171</v>
+        <v>0.17738252162458</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.19315539990012</v>
+        <v>0.192206035273382</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.182204433022843</v>
+        <v>0.182447949823553</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.220105537285106</v>
+        <v>0.21996811635111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.260525863340337</v>
+        <v>0.26011188683645</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.332040792593832</v>
+        <v>0.332584440641124</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.475861021629633</v>
+        <v>0.475987650564061</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.503255885804954</v>
+        <v>0.50242810943789</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.369539951580009</v>
+        <v>0.368592936570087</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.281217073276121</v>
+        <v>0.2801979943812</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.265412556698247</v>
+        <v>0.264824480633532</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.259472697425281</v>
+        <v>0.260863227353869</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.23647515922722</v>
+        <v>0.239673625136732</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.172101957765342</v>
+        <v>0.174845441412943</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.12057592475221</v>
+        <v>0.122008117829059</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.124910896214847</v>
+        <v>0.125152271321986</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.123875042235722</v>
+        <v>0.123315020766659</v>
       </c>
     </row>
     <row r="24">

</xml_diff>